<commit_message>
feat: envia email de confirmacao para tecnicos Mateos e Zanella sem botao de baixa
</commit_message>
<xml_diff>
--- a/data/Base Instalada.xlsx
+++ b/data/Base Instalada.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30309"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maquinascomprint-my.sharepoint.com/personal/ricardo_almeida_comprint_com_br/Documents/PROJETOS/OUTROS/Programação/chatbot-whatsapp-estoque/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="463" documentId="8_{51F1F06D-6D0B-4FE8-9AF7-39931DF9B484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B74CCCFB-9025-4911-9635-E3C3B97009EF}"/>
+  <xr:revisionPtr revIDLastSave="464" documentId="8_{51F1F06D-6D0B-4FE8-9AF7-39931DF9B484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8809713-4E18-4D4C-B370-A82EE7544C86}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FA3517F6-4E5E-4958-9700-7C1440F86859}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FA3517F6-4E5E-4958-9700-7C1440F86859}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="1" r:id="rId1"/>
@@ -660,7 +660,7 @@
     <numFmt numFmtId="164" formatCode="#,###,###,##0.00###"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1212,27 +1212,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385B57CD-294C-4E76-82E5-66AB1487D8F3}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O109"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" style="32" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.26953125" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="32" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.453125" style="7" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="33" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.1796875" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.453125" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.26953125" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.26953125" style="7" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" style="7" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.26953125" style="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1">
+    <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
@@ -1279,7 +1280,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -1294,11 +1295,11 @@
       </c>
       <c r="E2" s="13">
         <f t="shared" ref="E2:E33" ca="1" si="0">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F2" s="11">
         <f t="shared" ref="F2:F33" ca="1" si="1">D2-E2</f>
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>16</v>
@@ -1323,7 +1324,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -1338,11 +1339,11 @@
       </c>
       <c r="E3" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F3" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>21</v>
@@ -1367,7 +1368,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1382,11 +1383,11 @@
       </c>
       <c r="E4" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F4" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>22</v>
@@ -1411,7 +1412,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -1426,11 +1427,11 @@
       </c>
       <c r="E5" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F5" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>23</v>
@@ -1455,7 +1456,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -1470,11 +1471,11 @@
       </c>
       <c r="E6" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F6" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>26</v>
@@ -1499,7 +1500,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
@@ -1514,11 +1515,11 @@
       </c>
       <c r="E7" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>23</v>
@@ -1543,7 +1544,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -1558,11 +1559,11 @@
       </c>
       <c r="E8" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F8" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-158</v>
+        <v>-162</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>29</v>
@@ -1587,7 +1588,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -1602,11 +1603,11 @@
       </c>
       <c r="E9" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F9" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-395</v>
+        <v>-399</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>22</v>
@@ -1629,7 +1630,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -1644,11 +1645,11 @@
       </c>
       <c r="E10" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>31</v>
@@ -1671,7 +1672,7 @@
       <c r="N10" s="13"/>
       <c r="O10" s="19"/>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>30</v>
       </c>
@@ -1686,11 +1687,11 @@
       </c>
       <c r="E11" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F11" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>32</v>
@@ -1715,7 +1716,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>33</v>
       </c>
@@ -1730,11 +1731,11 @@
       </c>
       <c r="E12" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F12" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>34</v>
@@ -1760,7 +1761,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>37</v>
       </c>
@@ -1775,11 +1776,11 @@
       </c>
       <c r="E13" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F13" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>38</v>
@@ -1805,7 +1806,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>40</v>
       </c>
@@ -1820,11 +1821,11 @@
       </c>
       <c r="E14" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F14" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>16</v>
@@ -1848,7 +1849,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>42</v>
       </c>
@@ -1863,11 +1864,11 @@
       </c>
       <c r="E15" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F15" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>26</v>
@@ -1893,7 +1894,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
         <v>45</v>
       </c>
@@ -1908,11 +1909,11 @@
       </c>
       <c r="E16" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F16" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G16" s="12" t="s">
         <v>46</v>
@@ -1936,7 +1937,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
         <v>48</v>
       </c>
@@ -1951,11 +1952,11 @@
       </c>
       <c r="E17" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F17" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>49</v>
@@ -1979,7 +1980,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
         <v>50</v>
       </c>
@@ -1994,11 +1995,11 @@
       </c>
       <c r="E18" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F18" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="G18" s="12" t="s">
         <v>16</v>
@@ -2022,7 +2023,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
         <v>52</v>
       </c>
@@ -2037,11 +2038,11 @@
       </c>
       <c r="E19" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>26</v>
@@ -2065,7 +2066,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
         <v>53</v>
       </c>
@@ -2080,11 +2081,11 @@
       </c>
       <c r="E20" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F20" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G20" s="12" t="s">
         <v>16</v>
@@ -2108,7 +2109,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
         <v>54</v>
       </c>
@@ -2123,11 +2124,11 @@
       </c>
       <c r="E21" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F21" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G21" s="12" t="s">
         <v>31</v>
@@ -2152,7 +2153,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
         <v>55</v>
       </c>
@@ -2167,11 +2168,11 @@
       </c>
       <c r="E22" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F22" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G22" s="12" t="s">
         <v>32</v>
@@ -2196,7 +2197,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
         <v>56</v>
       </c>
@@ -2211,11 +2212,11 @@
       </c>
       <c r="E23" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F23" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-16</v>
+        <v>-20</v>
       </c>
       <c r="G23" s="12" t="s">
         <v>38</v>
@@ -2240,7 +2241,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="23" t="s">
         <v>58</v>
       </c>
@@ -2255,11 +2256,11 @@
       </c>
       <c r="E24" s="26">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F24" s="27">
         <f t="shared" ca="1" si="1"/>
-        <v>-16</v>
+        <v>-20</v>
       </c>
       <c r="G24" s="31" t="s">
         <v>59</v>
@@ -2286,7 +2287,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="23" t="s">
         <v>58</v>
       </c>
@@ -2301,11 +2302,11 @@
       </c>
       <c r="E25" s="26">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F25" s="27">
         <f t="shared" ca="1" si="1"/>
-        <v>-16</v>
+        <v>-20</v>
       </c>
       <c r="G25" s="31" t="s">
         <v>59</v>
@@ -2332,7 +2333,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>58</v>
       </c>
@@ -2347,11 +2348,11 @@
       </c>
       <c r="E26" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F26" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G26" s="12" t="s">
         <v>34</v>
@@ -2378,7 +2379,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
         <v>61</v>
       </c>
@@ -2393,11 +2394,11 @@
       </c>
       <c r="E27" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F27" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="G27" s="12" t="s">
         <v>34</v>
@@ -2424,7 +2425,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:15" s="30" customFormat="1">
+    <row r="28" spans="1:15" s="30" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
         <v>62</v>
       </c>
@@ -2439,11 +2440,11 @@
       </c>
       <c r="E28" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>5282</v>
+        <v>5278</v>
       </c>
       <c r="G28" s="12" t="s">
         <v>63</v>
@@ -2467,7 +2468,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:15" s="30" customFormat="1">
+    <row r="29" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>62</v>
       </c>
@@ -2482,11 +2483,11 @@
       </c>
       <c r="E29" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F29" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G29" s="12" t="s">
         <v>32</v>
@@ -2511,7 +2512,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
         <v>65</v>
       </c>
@@ -2526,11 +2527,11 @@
       </c>
       <c r="E30" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F30" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G30" s="12" t="s">
         <v>66</v>
@@ -2555,7 +2556,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" s="23" t="s">
         <v>67</v>
       </c>
@@ -2570,11 +2571,11 @@
       </c>
       <c r="E31" s="26">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F31" s="27">
         <f t="shared" ca="1" si="1"/>
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="G31" s="31" t="s">
         <v>16</v>
@@ -2599,7 +2600,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="14.25" customHeight="1">
+    <row r="32" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
         <v>68</v>
       </c>
@@ -2614,11 +2615,11 @@
       </c>
       <c r="E32" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F32" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G32" s="12" t="s">
         <v>31</v>
@@ -2643,7 +2644,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>69</v>
       </c>
@@ -2658,11 +2659,11 @@
       </c>
       <c r="E33" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F33" s="11">
         <f t="shared" ca="1" si="1"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G33" s="12" t="s">
         <v>22</v>
@@ -2687,7 +2688,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
         <v>70</v>
       </c>
@@ -2702,11 +2703,11 @@
       </c>
       <c r="E34" s="13">
         <f t="shared" ref="E34:E68" ca="1" si="4">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F34" s="11">
         <f t="shared" ref="F34:F65" ca="1" si="5">D34-E34</f>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G34" s="12" t="s">
         <v>21</v>
@@ -2731,7 +2732,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
         <v>71</v>
       </c>
@@ -2746,11 +2747,11 @@
       </c>
       <c r="E35" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F35" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="G35" s="12" t="s">
         <v>16</v>
@@ -2775,7 +2776,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:15" s="30" customFormat="1" ht="15" customHeight="1">
+    <row r="36" spans="1:15" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
         <v>72</v>
       </c>
@@ -2790,11 +2791,11 @@
       </c>
       <c r="E36" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F36" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="G36" s="12" t="s">
         <v>73</v>
@@ -2818,7 +2819,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
         <v>72</v>
       </c>
@@ -2833,11 +2834,11 @@
       </c>
       <c r="E37" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F37" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="G37" s="12" t="s">
         <v>75</v>
@@ -2861,7 +2862,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
         <v>76</v>
       </c>
@@ -2876,11 +2877,11 @@
       </c>
       <c r="E38" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F38" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-13</v>
+        <v>-17</v>
       </c>
       <c r="G38" s="12" t="s">
         <v>73</v>
@@ -2905,7 +2906,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
         <v>77</v>
       </c>
@@ -2920,11 +2921,11 @@
       </c>
       <c r="E39" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F39" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G39" s="12" t="s">
         <v>31</v>
@@ -2949,7 +2950,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:15">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
         <v>77</v>
       </c>
@@ -2964,11 +2965,11 @@
       </c>
       <c r="E40" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F40" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G40" s="12" t="s">
         <v>78</v>
@@ -2993,7 +2994,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:15">
+    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>79</v>
       </c>
@@ -3008,11 +3009,11 @@
       </c>
       <c r="E41" s="26">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F41" s="27">
         <f t="shared" ca="1" si="5"/>
-        <v>1360</v>
+        <v>1356</v>
       </c>
       <c r="G41" s="31" t="s">
         <v>80</v>
@@ -3036,7 +3037,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:15">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
         <v>83</v>
       </c>
@@ -3051,11 +3052,11 @@
       </c>
       <c r="E42" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F42" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G42" s="12" t="s">
         <v>31</v>
@@ -3080,7 +3081,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="1:15">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A43" s="8" t="s">
         <v>83</v>
       </c>
@@ -3095,11 +3096,11 @@
       </c>
       <c r="E43" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F43" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G43" s="12" t="s">
         <v>32</v>
@@ -3124,7 +3125,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="1:15" s="30" customFormat="1">
+    <row r="44" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
         <v>84</v>
       </c>
@@ -3139,11 +3140,11 @@
       </c>
       <c r="E44" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F44" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G44" s="12" t="s">
         <v>85</v>
@@ -3168,7 +3169,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="1:15">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A45" s="8" t="s">
         <v>86</v>
       </c>
@@ -3183,11 +3184,11 @@
       </c>
       <c r="E45" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F45" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G45" s="12" t="s">
         <v>31</v>
@@ -3212,7 +3213,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:15">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A46" s="8" t="s">
         <v>87</v>
       </c>
@@ -3227,11 +3228,11 @@
       </c>
       <c r="E46" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F46" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="G46" s="12" t="s">
         <v>16</v>
@@ -3256,7 +3257,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:15">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A47" s="8" t="s">
         <v>88</v>
       </c>
@@ -3271,11 +3272,11 @@
       </c>
       <c r="E47" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F47" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G47" s="12" t="s">
         <v>21</v>
@@ -3300,7 +3301,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:15">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A48" s="8" t="s">
         <v>89</v>
       </c>
@@ -3315,11 +3316,11 @@
       </c>
       <c r="E48" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F48" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G48" s="12" t="s">
         <v>63</v>
@@ -3346,7 +3347,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:15">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A49" s="8" t="s">
         <v>90</v>
       </c>
@@ -3361,11 +3362,11 @@
       </c>
       <c r="E49" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F49" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G49" s="12" t="s">
         <v>63</v>
@@ -3390,7 +3391,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:15">
+    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="8" t="s">
         <v>91</v>
       </c>
@@ -3405,11 +3406,11 @@
       </c>
       <c r="E50" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F50" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G50" s="12" t="s">
         <v>26</v>
@@ -3436,7 +3437,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="1:15">
+    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="8" t="s">
         <v>91</v>
       </c>
@@ -3451,11 +3452,11 @@
       </c>
       <c r="E51" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F51" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G51" s="12" t="s">
         <v>22</v>
@@ -3482,7 +3483,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:15">
+    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="8" t="s">
         <v>91</v>
       </c>
@@ -3497,11 +3498,11 @@
       </c>
       <c r="E52" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F52" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="G52" s="12" t="s">
         <v>16</v>
@@ -3528,7 +3529,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:15" s="30" customFormat="1">
+    <row r="53" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="8" t="s">
         <v>93</v>
       </c>
@@ -3543,11 +3544,11 @@
       </c>
       <c r="E53" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F53" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G53" s="12" t="s">
         <v>78</v>
@@ -3572,7 +3573,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="54" spans="1:15" s="30" customFormat="1">
+    <row r="54" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="8" t="s">
         <v>94</v>
       </c>
@@ -3587,11 +3588,11 @@
       </c>
       <c r="E54" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F54" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G54" s="12" t="s">
         <v>63</v>
@@ -3616,7 +3617,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:15">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A55" s="8" t="s">
         <v>95</v>
       </c>
@@ -3631,11 +3632,11 @@
       </c>
       <c r="E55" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F55" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G55" s="12" t="s">
         <v>22</v>
@@ -3660,7 +3661,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:15">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A56" s="8" t="s">
         <v>96</v>
       </c>
@@ -3675,11 +3676,11 @@
       </c>
       <c r="E56" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F56" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G56" s="12" t="s">
         <v>97</v>
@@ -3704,7 +3705,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:15">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A57" s="8" t="s">
         <v>96</v>
       </c>
@@ -3719,11 +3720,11 @@
       </c>
       <c r="E57" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F57" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G57" s="12" t="s">
         <v>63</v>
@@ -3748,7 +3749,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A58" s="8" t="s">
         <v>98</v>
       </c>
@@ -3763,11 +3764,11 @@
       </c>
       <c r="E58" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F58" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G58" s="12" t="s">
         <v>31</v>
@@ -3792,7 +3793,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="59" spans="1:15">
+    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="8" t="s">
         <v>99</v>
       </c>
@@ -3807,11 +3808,11 @@
       </c>
       <c r="E59" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F59" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G59" s="12" t="s">
         <v>34</v>
@@ -3835,7 +3836,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A60" s="8" t="s">
         <v>101</v>
       </c>
@@ -3850,11 +3851,11 @@
       </c>
       <c r="E60" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F60" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G60" s="12" t="s">
         <v>32</v>
@@ -3879,7 +3880,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A61" s="8" t="s">
         <v>102</v>
       </c>
@@ -3894,11 +3895,11 @@
       </c>
       <c r="E61" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F61" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-197</v>
+        <v>-201</v>
       </c>
       <c r="G61" s="12" t="s">
         <v>66</v>
@@ -3923,7 +3924,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:15">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A62" s="8" t="s">
         <v>103</v>
       </c>
@@ -3938,11 +3939,11 @@
       </c>
       <c r="E62" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F62" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G62" s="12" t="s">
         <v>104</v>
@@ -3967,7 +3968,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="1:15">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A63" s="8" t="s">
         <v>105</v>
       </c>
@@ -3982,11 +3983,11 @@
       </c>
       <c r="E63" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F63" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G63" s="12" t="s">
         <v>66</v>
@@ -4011,7 +4012,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:15">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A64" s="23" t="s">
         <v>105</v>
       </c>
@@ -4026,11 +4027,11 @@
       </c>
       <c r="E64" s="26">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F64" s="27">
         <f t="shared" ca="1" si="5"/>
-        <v>-137</v>
+        <v>-141</v>
       </c>
       <c r="G64" s="31" t="s">
         <v>16</v>
@@ -4055,7 +4056,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:15">
+    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="8" t="s">
         <v>106</v>
       </c>
@@ -4070,11 +4071,11 @@
       </c>
       <c r="E65" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F65" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>-16</v>
+        <v>-20</v>
       </c>
       <c r="G65" s="12" t="s">
         <v>63</v>
@@ -4098,7 +4099,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="66" spans="1:15">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A66" s="8" t="s">
         <v>107</v>
       </c>
@@ -4113,11 +4114,11 @@
       </c>
       <c r="E66" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F66" s="11">
-        <f t="shared" ref="F66:F97" ca="1" si="7">D66-E66</f>
-        <v>-2023</v>
+        <f t="shared" ref="F66:F68" ca="1" si="7">D66-E66</f>
+        <v>-2027</v>
       </c>
       <c r="G66" s="12" t="s">
         <v>31</v>
@@ -4142,7 +4143,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="67" spans="1:15">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A67" s="8" t="s">
         <v>107</v>
       </c>
@@ -4157,11 +4158,11 @@
       </c>
       <c r="E67" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F67" s="11">
         <f t="shared" ca="1" si="7"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G67" s="12" t="s">
         <v>63</v>
@@ -4186,7 +4187,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="68" spans="1:15" s="30" customFormat="1">
+    <row r="68" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="8" t="s">
         <v>108</v>
       </c>
@@ -4201,11 +4202,11 @@
       </c>
       <c r="E68" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F68" s="11">
         <f t="shared" ca="1" si="7"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G68" s="12" t="s">
         <v>32</v>
@@ -4230,7 +4231,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="69" spans="1:15">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A69" s="8" t="s">
         <v>109</v>
       </c>
@@ -4253,7 +4254,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="70" spans="1:15">
+    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="23" t="s">
         <v>109</v>
       </c>
@@ -4268,11 +4269,11 @@
       </c>
       <c r="E70" s="25">
         <f t="shared" ref="E70:E103" ca="1" si="8">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F70" s="27">
         <f t="shared" ref="F70:F103" ca="1" si="9">D70-E70</f>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G70" s="31" t="s">
         <v>22</v>
@@ -4295,7 +4296,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" spans="1:15">
+    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="8" t="s">
         <v>110</v>
       </c>
@@ -4310,11 +4311,11 @@
       </c>
       <c r="E71" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F71" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G71" s="12" t="s">
         <v>34</v>
@@ -4340,7 +4341,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="72" spans="1:15">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A72" s="8" t="s">
         <v>113</v>
       </c>
@@ -4355,11 +4356,11 @@
       </c>
       <c r="E72" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F72" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G72" s="12" t="s">
         <v>66</v>
@@ -4382,7 +4383,7 @@
       <c r="N72" s="14"/>
       <c r="O72" s="19"/>
     </row>
-    <row r="73" spans="1:15">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A73" s="8" t="s">
         <v>113</v>
       </c>
@@ -4397,11 +4398,11 @@
       </c>
       <c r="E73" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F73" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G73" s="12" t="s">
         <v>22</v>
@@ -4426,7 +4427,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="74" spans="1:15">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A74" s="8" t="s">
         <v>114</v>
       </c>
@@ -4441,11 +4442,11 @@
       </c>
       <c r="E74" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F74" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="G74" s="12" t="s">
         <v>32</v>
@@ -4472,7 +4473,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="75" spans="1:15">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A75" s="8" t="s">
         <v>114</v>
       </c>
@@ -4487,11 +4488,11 @@
       </c>
       <c r="E75" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F75" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="G75" s="12" t="s">
         <v>85</v>
@@ -4518,7 +4519,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="1:15">
+    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="8" t="s">
         <v>116</v>
       </c>
@@ -4533,11 +4534,11 @@
       </c>
       <c r="E76" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F76" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G76" s="12" t="s">
         <v>23</v>
@@ -4564,7 +4565,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="77" spans="1:15">
+    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="8" t="s">
         <v>118</v>
       </c>
@@ -4579,11 +4580,11 @@
       </c>
       <c r="E77" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F77" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="G77" s="12" t="s">
         <v>119</v>
@@ -4609,7 +4610,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="78" spans="1:15">
+    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="8" t="s">
         <v>122</v>
       </c>
@@ -4624,11 +4625,11 @@
       </c>
       <c r="E78" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F78" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G78" s="12" t="s">
         <v>34</v>
@@ -4653,7 +4654,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="79" spans="1:15">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A79" s="8" t="s">
         <v>124</v>
       </c>
@@ -4668,11 +4669,11 @@
       </c>
       <c r="E79" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F79" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G79" s="12" t="s">
         <v>66</v>
@@ -4697,7 +4698,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="80" spans="1:15">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A80" s="8" t="s">
         <v>124</v>
       </c>
@@ -4712,11 +4713,11 @@
       </c>
       <c r="E80" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F80" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G80" s="12" t="s">
         <v>26</v>
@@ -4741,7 +4742,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="81" spans="1:15">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A81" s="8" t="s">
         <v>124</v>
       </c>
@@ -4756,11 +4757,11 @@
       </c>
       <c r="E81" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F81" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G81" s="12" t="s">
         <v>26</v>
@@ -4785,7 +4786,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="82" spans="1:15">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A82" s="8" t="s">
         <v>125</v>
       </c>
@@ -4800,11 +4801,11 @@
       </c>
       <c r="E82" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F82" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G82" s="12" t="s">
         <v>22</v>
@@ -4829,7 +4830,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="83" spans="1:15">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A83" s="8" t="s">
         <v>125</v>
       </c>
@@ -4844,11 +4845,11 @@
       </c>
       <c r="E83" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F83" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G83" s="12" t="s">
         <v>16</v>
@@ -4873,7 +4874,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="84" spans="1:15">
+    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="8" t="s">
         <v>126</v>
       </c>
@@ -4888,11 +4889,11 @@
       </c>
       <c r="E84" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F84" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="G84" s="12" t="s">
         <v>75</v>
@@ -4914,7 +4915,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="85" spans="1:15">
+    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="8" t="s">
         <v>126</v>
       </c>
@@ -4929,11 +4930,11 @@
       </c>
       <c r="E85" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F85" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G85" s="12" t="s">
         <v>34</v>
@@ -4957,7 +4958,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:15">
+    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="8" t="s">
         <v>126</v>
       </c>
@@ -4972,11 +4973,11 @@
       </c>
       <c r="E86" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F86" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G86" s="12" t="s">
         <v>73</v>
@@ -5000,7 +5001,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="87" spans="1:15">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A87" s="10" t="s">
         <v>130</v>
       </c>
@@ -5015,11 +5016,11 @@
       </c>
       <c r="E87" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F87" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G87" s="12" t="s">
         <v>21</v>
@@ -5042,7 +5043,7 @@
       <c r="N87" s="14"/>
       <c r="O87" s="19"/>
     </row>
-    <row r="88" spans="1:15">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A88" s="10" t="s">
         <v>131</v>
       </c>
@@ -5057,11 +5058,11 @@
       </c>
       <c r="E88" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F88" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G88" s="12" t="s">
         <v>31</v>
@@ -5086,7 +5087,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="89" spans="1:15">
+    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="10" t="s">
         <v>132</v>
       </c>
@@ -5101,11 +5102,11 @@
       </c>
       <c r="E89" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F89" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="G89" s="12" t="s">
         <v>104</v>
@@ -5127,7 +5128,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="90" spans="1:15">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A90" s="8" t="s">
         <v>134</v>
       </c>
@@ -5142,11 +5143,11 @@
       </c>
       <c r="E90" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F90" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="G90" s="12" t="s">
         <v>22</v>
@@ -5171,7 +5172,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="91" spans="1:15">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A91" s="8" t="s">
         <v>134</v>
       </c>
@@ -5186,11 +5187,11 @@
       </c>
       <c r="E91" s="13">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F91" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="G91" s="12" t="s">
         <v>16</v>
@@ -5213,7 +5214,7 @@
       <c r="N91" s="14"/>
       <c r="O91" s="19"/>
     </row>
-    <row r="92" spans="1:15">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A92" s="8" t="s">
         <v>135</v>
       </c>
@@ -5228,11 +5229,11 @@
       </c>
       <c r="E92" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F92" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G92" s="12" t="s">
         <v>136</v>
@@ -5257,7 +5258,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="93" spans="1:15">
+    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="23" t="s">
         <v>137</v>
       </c>
@@ -5272,11 +5273,11 @@
       </c>
       <c r="E93" s="26">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F93" s="27">
         <f t="shared" ca="1" si="9"/>
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="G93" s="31" t="s">
         <v>26</v>
@@ -5303,7 +5304,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="1:15">
+    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="23" t="s">
         <v>137</v>
       </c>
@@ -5318,11 +5319,11 @@
       </c>
       <c r="E94" s="26">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F94" s="27">
         <f t="shared" ca="1" si="9"/>
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="G94" s="31" t="s">
         <v>16</v>
@@ -5349,7 +5350,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="95" spans="1:15">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A95" s="8" t="s">
         <v>138</v>
       </c>
@@ -5364,11 +5365,11 @@
       </c>
       <c r="E95" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F95" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G95" s="12" t="s">
         <v>31</v>
@@ -5393,7 +5394,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="96" spans="1:15" s="30" customFormat="1">
+    <row r="96" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A96" s="23" t="s">
         <v>139</v>
       </c>
@@ -5408,11 +5409,11 @@
       </c>
       <c r="E96" s="25">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F96" s="27">
         <f t="shared" ca="1" si="9"/>
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="G96" s="31" t="s">
         <v>32</v>
@@ -5437,7 +5438,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="97" spans="1:15" ht="14.25" customHeight="1">
+    <row r="97" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="8" t="s">
         <v>140</v>
       </c>
@@ -5452,11 +5453,11 @@
       </c>
       <c r="E97" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F97" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G97" s="12" t="s">
         <v>21</v>
@@ -5481,7 +5482,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="98" spans="1:15">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A98" s="8" t="s">
         <v>141</v>
       </c>
@@ -5496,11 +5497,11 @@
       </c>
       <c r="E98" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F98" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="G98" s="12" t="s">
         <v>85</v>
@@ -5525,7 +5526,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="99" spans="1:15">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A99" s="8" t="s">
         <v>142</v>
       </c>
@@ -5540,11 +5541,11 @@
       </c>
       <c r="E99" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F99" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G99" s="12" t="s">
         <v>31</v>
@@ -5569,7 +5570,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="100" spans="1:15">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A100" s="8" t="s">
         <v>143</v>
       </c>
@@ -5584,11 +5585,11 @@
       </c>
       <c r="E100" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F100" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G100" s="12" t="s">
         <v>104</v>
@@ -5613,7 +5614,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="101" spans="1:15">
+    <row r="101" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="8" t="s">
         <v>144</v>
       </c>
@@ -5628,11 +5629,11 @@
       </c>
       <c r="E101" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F101" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="G101" s="12" t="s">
         <v>104</v>
@@ -5657,7 +5658,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="102" spans="1:15">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A102" s="8" t="s">
         <v>146</v>
       </c>
@@ -5672,11 +5673,11 @@
       </c>
       <c r="E102" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F102" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="G102" s="12" t="s">
         <v>16</v>
@@ -5701,7 +5702,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="103" spans="1:15" s="30" customFormat="1">
+    <row r="103" spans="1:15" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="8" t="s">
         <v>147</v>
       </c>
@@ -5716,11 +5717,11 @@
       </c>
       <c r="E103" s="14">
         <f t="shared" ca="1" si="8"/>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F103" s="11">
         <f t="shared" ca="1" si="9"/>
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="G103" s="12" t="s">
         <v>148</v>
@@ -5745,7 +5746,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="104" spans="1:15">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A104" s="8" t="s">
         <v>149</v>
       </c>
@@ -5770,7 +5771,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="105" spans="1:15">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A105" s="8" t="s">
         <v>150</v>
       </c>
@@ -5785,11 +5786,11 @@
       </c>
       <c r="E105" s="14">
         <f ca="1">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F105" s="11">
         <f ca="1">D105-E105</f>
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G105" s="12" t="s">
         <v>38</v>
@@ -5812,7 +5813,7 @@
       <c r="N105" s="14"/>
       <c r="O105" s="19"/>
     </row>
-    <row r="106" spans="1:15">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A106" s="8" t="s">
         <v>150</v>
       </c>
@@ -5827,11 +5828,11 @@
       </c>
       <c r="E106" s="14">
         <f ca="1">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F106" s="11">
         <f ca="1">D106-E106</f>
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="G106" s="12" t="s">
         <v>29</v>
@@ -5856,7 +5857,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="107" spans="1:15">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A107" s="8" t="s">
         <v>151</v>
       </c>
@@ -5871,11 +5872,11 @@
       </c>
       <c r="E107" s="14">
         <f ca="1">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F107" s="11">
         <f ca="1">D107-E107</f>
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="G107" s="12" t="s">
         <v>34</v>
@@ -5900,7 +5901,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="108" spans="1:15">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A108" s="8" t="s">
         <v>152</v>
       </c>
@@ -5915,11 +5916,11 @@
       </c>
       <c r="E108" s="14">
         <f ca="1">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F108" s="11">
         <f ca="1">D108-E108</f>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G108" s="12" t="s">
         <v>136</v>
@@ -5944,7 +5945,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="109" spans="1:15">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A109" s="8" t="s">
         <v>152</v>
       </c>
@@ -5959,11 +5960,11 @@
       </c>
       <c r="E109" s="14">
         <f ca="1">TODAY()</f>
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="F109" s="11">
         <f ca="1">D109-E109</f>
-        <v>-2023</v>
+        <v>-2027</v>
       </c>
       <c r="G109" s="12" t="s">
         <v>31</v>
@@ -5990,6 +5991,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:N109" xr:uid="{385B57CD-294C-4E76-82E5-66AB1487D8F3}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="AVULSO"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N109">
       <sortCondition ref="A1:A109"/>
     </sortState>
@@ -6001,25 +6007,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C0B4294-6308-408D-A7E0-6148B7D61ACB}">
   <dimension ref="A1:N38"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" style="7" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="9.7265625" customWidth="1"/>
     <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" style="7" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" style="7" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.26953125" style="7" customWidth="1"/>
+    <col min="9" max="9" width="15.54296875" style="7" customWidth="1"/>
+    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="4" customFormat="1">
+    <row r="1" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6063,7 +6069,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>158</v>
       </c>
@@ -6101,7 +6107,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>163</v>
       </c>
@@ -6139,7 +6145,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>165</v>
       </c>
@@ -6177,7 +6183,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>167</v>
       </c>
@@ -6215,7 +6221,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>168</v>
       </c>
@@ -6253,7 +6259,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>169</v>
       </c>
@@ -6291,7 +6297,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>171</v>
       </c>
@@ -6329,7 +6335,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>172</v>
       </c>
@@ -6367,7 +6373,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>173</v>
       </c>
@@ -6405,7 +6411,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>174</v>
       </c>
@@ -6443,7 +6449,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>68</v>
       </c>
@@ -6481,7 +6487,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>69</v>
       </c>
@@ -6519,7 +6525,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>175</v>
       </c>
@@ -6557,7 +6563,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>176</v>
       </c>
@@ -6595,7 +6601,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>178</v>
       </c>
@@ -6633,7 +6639,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>179</v>
       </c>
@@ -6671,7 +6677,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>181</v>
       </c>
@@ -6709,7 +6715,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>182</v>
       </c>
@@ -6747,7 +6753,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>183</v>
       </c>
@@ -6785,7 +6791,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>184</v>
       </c>
@@ -6823,7 +6829,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>87</v>
       </c>
@@ -6861,7 +6867,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>186</v>
       </c>
@@ -6899,7 +6905,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>188</v>
       </c>
@@ -6937,7 +6943,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>189</v>
       </c>
@@ -6975,7 +6981,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>190</v>
       </c>
@@ -7013,7 +7019,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>191</v>
       </c>
@@ -7051,7 +7057,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>193</v>
       </c>
@@ -7089,7 +7095,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>194</v>
       </c>
@@ -7127,7 +7133,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>108</v>
       </c>
@@ -7165,7 +7171,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>195</v>
       </c>
@@ -7203,7 +7209,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>196</v>
       </c>
@@ -7241,7 +7247,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>197</v>
       </c>
@@ -7279,7 +7285,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>199</v>
       </c>
@@ -7317,7 +7323,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>200</v>
       </c>
@@ -7355,7 +7361,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>201</v>
       </c>
@@ -7393,7 +7399,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>202</v>
       </c>
@@ -7431,7 +7437,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>202</v>
       </c>

</xml_diff>

<commit_message>
feat: adicionar botão sair no painel kanban
</commit_message>
<xml_diff>
--- a/data/Base Instalada.xlsx
+++ b/data/Base Instalada.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maquinascomprint-my.sharepoint.com/personal/ricardo_almeida_comprint_com_br/Documents/PROJETOS/OUTROS/Programação/chatbot-whatsapp-estoque/data/"/>
@@ -328,6 +328,12 @@
     <t>IPSIS</t>
   </si>
   <si>
+    <t>HP INDIGO 18K</t>
+  </si>
+  <si>
+    <t>03 MESES DE MÃO DE OBRA (ATÉ 31/10/26)</t>
+  </si>
+  <si>
     <t>JM EMBALAGENS</t>
   </si>
   <si>
@@ -385,6 +391,12 @@
     <t>OUTLABEL</t>
   </si>
   <si>
+    <t>03 MESES DE MÃO DE OBRA</t>
+  </si>
+  <si>
+    <t>AGUARDANDO ENTREGA</t>
+  </si>
+  <si>
     <t xml:space="preserve">P+E </t>
   </si>
   <si>
@@ -400,9 +412,6 @@
     <t xml:space="preserve">PIGMA    </t>
   </si>
   <si>
-    <t>HP INDIGO 18K</t>
-  </si>
-  <si>
     <t>SERVIÇOS ATÉ 27/11/27</t>
   </si>
   <si>
@@ -650,15 +659,6 @@
   </si>
   <si>
     <t>ULTRAPRESS EDITORA E GRAFICA</t>
-  </si>
-  <si>
-    <t>03 MESES DE MÃO DE OBRA (ATÉ 31/10/26)</t>
-  </si>
-  <si>
-    <t>03 MESES DE MÃO DE OBRA</t>
-  </si>
-  <si>
-    <t>AGUARDANDO ENTREGA</t>
   </si>
 </sst>
 </file>
@@ -669,7 +669,7 @@
     <numFmt numFmtId="164" formatCode="#,###,###,##0.00###"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1395,26 +1395,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385B57CD-294C-4E76-82E5-66AB1487D8F3}">
   <dimension ref="A1:O110"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1796875" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.26953125" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.26953125" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.453125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" style="7" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="33" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.1796875" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.453125" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.26953125" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.26953125" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" style="7" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.26953125" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.28515625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:15" s="4" customFormat="1" ht="15" thickBot="1">
       <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15">
       <c r="A2" s="41" t="s">
         <v>14</v>
       </c>
@@ -1476,11 +1476,11 @@
       </c>
       <c r="E2" s="43">
         <f t="shared" ref="E2:E33" ca="1" si="0">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F2" s="44">
         <f t="shared" ref="F2:F33" ca="1" si="1">D2-E2</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" s="45" t="s">
         <v>16</v>
@@ -1505,7 +1505,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15">
       <c r="A3" s="28" t="s">
         <v>19</v>
       </c>
@@ -1520,11 +1520,11 @@
       </c>
       <c r="E3" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F3" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G3" s="16" t="s">
         <v>21</v>
@@ -1549,7 +1549,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15">
       <c r="A4" s="28" t="s">
         <v>19</v>
       </c>
@@ -1564,11 +1564,11 @@
       </c>
       <c r="E4" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F4" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G4" s="16" t="s">
         <v>22</v>
@@ -1593,7 +1593,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15">
       <c r="A5" s="28" t="s">
         <v>19</v>
       </c>
@@ -1608,11 +1608,11 @@
       </c>
       <c r="E5" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F5" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G5" s="16" t="s">
         <v>23</v>
@@ -1637,7 +1637,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15">
       <c r="A6" s="28" t="s">
         <v>25</v>
       </c>
@@ -1652,11 +1652,11 @@
       </c>
       <c r="E6" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F6" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G6" s="16" t="s">
         <v>26</v>
@@ -1681,7 +1681,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15">
       <c r="A7" s="28" t="s">
         <v>25</v>
       </c>
@@ -1696,11 +1696,11 @@
       </c>
       <c r="E7" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F7" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>23</v>
@@ -1725,7 +1725,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15">
       <c r="A8" s="28" t="s">
         <v>27</v>
       </c>
@@ -1740,11 +1740,11 @@
       </c>
       <c r="E8" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F8" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-165</v>
+        <v>-166</v>
       </c>
       <c r="G8" s="16" t="s">
         <v>29</v>
@@ -1769,7 +1769,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -1784,11 +1784,11 @@
       </c>
       <c r="E9" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F9" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-402</v>
+        <v>-403</v>
       </c>
       <c r="G9" s="16" t="s">
         <v>22</v>
@@ -1811,7 +1811,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15">
       <c r="A10" s="28" t="s">
         <v>30</v>
       </c>
@@ -1826,11 +1826,11 @@
       </c>
       <c r="E10" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F10" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>31</v>
@@ -1853,7 +1853,7 @@
       <c r="N10" s="11"/>
       <c r="O10" s="29"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15">
       <c r="A11" s="30" t="s">
         <v>30</v>
       </c>
@@ -1868,11 +1868,11 @@
       </c>
       <c r="E11" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F11" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G11" s="16" t="s">
         <v>32</v>
@@ -1897,7 +1897,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15">
       <c r="A12" s="30" t="s">
         <v>33</v>
       </c>
@@ -1912,11 +1912,11 @@
       </c>
       <c r="E12" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F12" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G12" s="16" t="s">
         <v>34</v>
@@ -1942,7 +1942,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15">
       <c r="A13" s="30" t="s">
         <v>37</v>
       </c>
@@ -1957,11 +1957,11 @@
       </c>
       <c r="E13" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F13" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>38</v>
@@ -1987,7 +1987,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15">
       <c r="A14" s="30" t="s">
         <v>40</v>
       </c>
@@ -2002,11 +2002,11 @@
       </c>
       <c r="E14" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F14" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>16</v>
@@ -2030,7 +2030,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15">
       <c r="A15" s="30" t="s">
         <v>42</v>
       </c>
@@ -2045,11 +2045,11 @@
       </c>
       <c r="E15" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F15" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G15" s="16" t="s">
         <v>26</v>
@@ -2075,7 +2075,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15">
       <c r="A16" s="30" t="s">
         <v>45</v>
       </c>
@@ -2090,11 +2090,11 @@
       </c>
       <c r="E16" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F16" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G16" s="16" t="s">
         <v>46</v>
@@ -2118,7 +2118,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15">
       <c r="A17" s="30" t="s">
         <v>48</v>
       </c>
@@ -2133,11 +2133,11 @@
       </c>
       <c r="E17" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F17" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>49</v>
@@ -2161,7 +2161,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15">
       <c r="A18" s="30" t="s">
         <v>50</v>
       </c>
@@ -2176,11 +2176,11 @@
       </c>
       <c r="E18" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F18" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="G18" s="16" t="s">
         <v>16</v>
@@ -2204,7 +2204,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15">
       <c r="A19" s="30" t="s">
         <v>52</v>
       </c>
@@ -2219,11 +2219,11 @@
       </c>
       <c r="E19" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F19" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G19" s="16" t="s">
         <v>26</v>
@@ -2247,7 +2247,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15">
       <c r="A20" s="30" t="s">
         <v>53</v>
       </c>
@@ -2262,11 +2262,11 @@
       </c>
       <c r="E20" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F20" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>16</v>
@@ -2290,7 +2290,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15">
       <c r="A21" s="30" t="s">
         <v>54</v>
       </c>
@@ -2305,11 +2305,11 @@
       </c>
       <c r="E21" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F21" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>31</v>
@@ -2334,7 +2334,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15">
       <c r="A22" s="30" t="s">
         <v>55</v>
       </c>
@@ -2349,11 +2349,11 @@
       </c>
       <c r="E22" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F22" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>32</v>
@@ -2378,7 +2378,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15">
       <c r="A23" s="30" t="s">
         <v>56</v>
       </c>
@@ -2393,11 +2393,11 @@
       </c>
       <c r="E23" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F23" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G23" s="16" t="s">
         <v>38</v>
@@ -2422,7 +2422,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15">
       <c r="A24" s="31" t="s">
         <v>58</v>
       </c>
@@ -2437,11 +2437,11 @@
       </c>
       <c r="E24" s="23">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F24" s="24">
         <f t="shared" ca="1" si="1"/>
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G24" s="25" t="s">
         <v>59</v>
@@ -2468,7 +2468,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15">
       <c r="A25" s="31" t="s">
         <v>58</v>
       </c>
@@ -2483,11 +2483,11 @@
       </c>
       <c r="E25" s="23">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F25" s="24">
         <f t="shared" ca="1" si="1"/>
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G25" s="25" t="s">
         <v>59</v>
@@ -2514,7 +2514,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15">
       <c r="A26" s="30" t="s">
         <v>58</v>
       </c>
@@ -2529,11 +2529,11 @@
       </c>
       <c r="E26" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F26" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G26" s="16" t="s">
         <v>34</v>
@@ -2560,7 +2560,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15">
       <c r="A27" s="30" t="s">
         <v>61</v>
       </c>
@@ -2575,11 +2575,11 @@
       </c>
       <c r="E27" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F27" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G27" s="16" t="s">
         <v>34</v>
@@ -2606,7 +2606,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" s="9" customFormat="1">
       <c r="A28" s="30" t="s">
         <v>62</v>
       </c>
@@ -2621,11 +2621,11 @@
       </c>
       <c r="E28" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F28" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>5275</v>
+        <v>5274</v>
       </c>
       <c r="G28" s="16" t="s">
         <v>63</v>
@@ -2649,7 +2649,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" s="9" customFormat="1">
       <c r="A29" s="30" t="s">
         <v>62</v>
       </c>
@@ -2664,11 +2664,11 @@
       </c>
       <c r="E29" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F29" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G29" s="16" t="s">
         <v>32</v>
@@ -2693,7 +2693,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15">
       <c r="A30" s="30" t="s">
         <v>65</v>
       </c>
@@ -2708,11 +2708,11 @@
       </c>
       <c r="E30" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F30" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G30" s="16" t="s">
         <v>66</v>
@@ -2737,7 +2737,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15">
       <c r="A31" s="31" t="s">
         <v>67</v>
       </c>
@@ -2752,11 +2752,11 @@
       </c>
       <c r="E31" s="23">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F31" s="24">
         <f t="shared" ca="1" si="1"/>
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G31" s="25" t="s">
         <v>16</v>
@@ -2781,7 +2781,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" ht="14.25" customHeight="1">
       <c r="A32" s="30" t="s">
         <v>68</v>
       </c>
@@ -2796,11 +2796,11 @@
       </c>
       <c r="E32" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F32" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G32" s="16" t="s">
         <v>31</v>
@@ -2825,7 +2825,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15">
       <c r="A33" s="28" t="s">
         <v>69</v>
       </c>
@@ -2840,11 +2840,11 @@
       </c>
       <c r="E33" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F33" s="15">
         <f t="shared" ca="1" si="1"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G33" s="16" t="s">
         <v>22</v>
@@ -2869,7 +2869,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15">
       <c r="A34" s="30" t="s">
         <v>70</v>
       </c>
@@ -2884,11 +2884,11 @@
       </c>
       <c r="E34" s="11">
         <f t="shared" ref="E34:E68" ca="1" si="4">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F34" s="15">
         <f t="shared" ref="F34:F65" ca="1" si="5">D34-E34</f>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G34" s="16" t="s">
         <v>21</v>
@@ -2913,7 +2913,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15">
       <c r="A35" s="30" t="s">
         <v>71</v>
       </c>
@@ -2928,11 +2928,11 @@
       </c>
       <c r="E35" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F35" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G35" s="16" t="s">
         <v>16</v>
@@ -2957,7 +2957,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:15" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" s="9" customFormat="1" ht="15" customHeight="1">
       <c r="A36" s="30" t="s">
         <v>72</v>
       </c>
@@ -2972,11 +2972,11 @@
       </c>
       <c r="E36" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F36" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G36" s="16" t="s">
         <v>73</v>
@@ -3000,7 +3000,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15">
       <c r="A37" s="30" t="s">
         <v>72</v>
       </c>
@@ -3015,11 +3015,11 @@
       </c>
       <c r="E37" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F37" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G37" s="16" t="s">
         <v>75</v>
@@ -3043,7 +3043,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15">
       <c r="A38" s="30" t="s">
         <v>76</v>
       </c>
@@ -3058,11 +3058,11 @@
       </c>
       <c r="E38" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F38" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-20</v>
+        <v>-21</v>
       </c>
       <c r="G38" s="16" t="s">
         <v>73</v>
@@ -3087,7 +3087,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15">
       <c r="A39" s="30" t="s">
         <v>77</v>
       </c>
@@ -3102,11 +3102,11 @@
       </c>
       <c r="E39" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F39" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G39" s="16" t="s">
         <v>31</v>
@@ -3131,7 +3131,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15">
       <c r="A40" s="30" t="s">
         <v>77</v>
       </c>
@@ -3146,11 +3146,11 @@
       </c>
       <c r="E40" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F40" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G40" s="16" t="s">
         <v>78</v>
@@ -3175,7 +3175,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15">
       <c r="A41" s="31" t="s">
         <v>79</v>
       </c>
@@ -3190,11 +3190,11 @@
       </c>
       <c r="E41" s="23">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F41" s="24">
         <f t="shared" ca="1" si="5"/>
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="G41" s="25" t="s">
         <v>80</v>
@@ -3218,7 +3218,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15">
       <c r="A42" s="30" t="s">
         <v>83</v>
       </c>
@@ -3233,11 +3233,11 @@
       </c>
       <c r="E42" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F42" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G42" s="16" t="s">
         <v>31</v>
@@ -3262,7 +3262,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15">
       <c r="A43" s="30" t="s">
         <v>83</v>
       </c>
@@ -3277,11 +3277,11 @@
       </c>
       <c r="E43" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F43" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G43" s="16" t="s">
         <v>32</v>
@@ -3306,7 +3306,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" s="9" customFormat="1">
       <c r="A44" s="30" t="s">
         <v>84</v>
       </c>
@@ -3321,11 +3321,11 @@
       </c>
       <c r="E44" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F44" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G44" s="16" t="s">
         <v>85</v>
@@ -3350,7 +3350,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:15">
       <c r="A45" s="30" t="s">
         <v>86</v>
       </c>
@@ -3365,11 +3365,11 @@
       </c>
       <c r="E45" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F45" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G45" s="16" t="s">
         <v>31</v>
@@ -3394,7 +3394,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15">
       <c r="A46" s="30" t="s">
         <v>87</v>
       </c>
@@ -3409,11 +3409,11 @@
       </c>
       <c r="E46" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F46" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G46" s="16" t="s">
         <v>16</v>
@@ -3438,7 +3438,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:15">
       <c r="A47" s="30" t="s">
         <v>88</v>
       </c>
@@ -3453,11 +3453,11 @@
       </c>
       <c r="E47" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F47" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G47" s="16" t="s">
         <v>21</v>
@@ -3482,7 +3482,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:15">
       <c r="A48" s="30" t="s">
         <v>89</v>
       </c>
@@ -3497,11 +3497,11 @@
       </c>
       <c r="E48" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F48" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G48" s="16" t="s">
         <v>63</v>
@@ -3528,7 +3528,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:15">
       <c r="A49" s="30" t="s">
         <v>90</v>
       </c>
@@ -3543,11 +3543,11 @@
       </c>
       <c r="E49" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F49" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G49" s="16" t="s">
         <v>63</v>
@@ -3572,7 +3572,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:15">
       <c r="A50" s="30" t="s">
         <v>91</v>
       </c>
@@ -3587,11 +3587,11 @@
       </c>
       <c r="E50" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F50" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G50" s="16" t="s">
         <v>26</v>
@@ -3618,7 +3618,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15">
       <c r="A51" s="30" t="s">
         <v>91</v>
       </c>
@@ -3633,11 +3633,11 @@
       </c>
       <c r="E51" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F51" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G51" s="16" t="s">
         <v>22</v>
@@ -3664,7 +3664,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:15">
       <c r="A52" s="30" t="s">
         <v>91</v>
       </c>
@@ -3679,11 +3679,11 @@
       </c>
       <c r="E52" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F52" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="G52" s="16" t="s">
         <v>16</v>
@@ -3710,7 +3710,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" s="9" customFormat="1">
       <c r="A53" s="30" t="s">
         <v>93</v>
       </c>
@@ -3725,11 +3725,11 @@
       </c>
       <c r="E53" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F53" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G53" s="16" t="s">
         <v>78</v>
@@ -3754,7 +3754,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="54" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:15" s="9" customFormat="1">
       <c r="A54" s="30" t="s">
         <v>94</v>
       </c>
@@ -3769,21 +3769,21 @@
       </c>
       <c r="E54" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F54" s="15">
         <f t="shared" ref="F54" ca="1" si="7">D54-E54</f>
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="G54" s="16" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="H54" s="18" t="str">
         <f t="shared" ref="H54" ca="1" si="8">IF(F54&lt;=0, "VENDA","CAREPACK")</f>
         <v>CAREPACK</v>
       </c>
       <c r="I54" s="18" t="s">
-        <v>203</v>
+        <v>96</v>
       </c>
       <c r="J54" s="15" t="s">
         <v>24</v>
@@ -3798,9 +3798,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15">
       <c r="A55" s="30" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>15</v>
@@ -3813,11 +3813,11 @@
       </c>
       <c r="E55" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F55" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G55" s="16" t="s">
         <v>22</v>
@@ -3842,9 +3842,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15">
       <c r="A56" s="30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B56" s="14" t="s">
         <v>15</v>
@@ -3857,14 +3857,14 @@
       </c>
       <c r="E56" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F56" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G56" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H56" s="18" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -3886,9 +3886,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15">
       <c r="A57" s="30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>15</v>
@@ -3901,11 +3901,11 @@
       </c>
       <c r="E57" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F57" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G57" s="16" t="s">
         <v>63</v>
@@ -3930,9 +3930,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15">
       <c r="A58" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B58" s="14" t="s">
         <v>15</v>
@@ -3945,11 +3945,11 @@
       </c>
       <c r="E58" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F58" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G58" s="16" t="s">
         <v>31</v>
@@ -3974,9 +3974,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15">
       <c r="A59" s="30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B59" s="20" t="s">
         <v>20</v>
@@ -3989,11 +3989,11 @@
       </c>
       <c r="E59" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F59" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G59" s="16" t="s">
         <v>34</v>
@@ -4002,7 +4002,7 @@
         <v>35</v>
       </c>
       <c r="I59" s="18" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J59" s="15" t="s">
         <v>24</v>
@@ -4017,9 +4017,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15">
       <c r="A60" s="30" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B60" s="14" t="s">
         <v>15</v>
@@ -4032,11 +4032,11 @@
       </c>
       <c r="E60" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F60" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G60" s="16" t="s">
         <v>32</v>
@@ -4061,9 +4061,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15">
       <c r="A61" s="30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B61" s="20" t="s">
         <v>20</v>
@@ -4076,11 +4076,11 @@
       </c>
       <c r="E61" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F61" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-204</v>
+        <v>-205</v>
       </c>
       <c r="G61" s="16" t="s">
         <v>66</v>
@@ -4105,9 +4105,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:15">
       <c r="A62" s="30" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B62" s="14" t="s">
         <v>15</v>
@@ -4120,14 +4120,14 @@
       </c>
       <c r="E62" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F62" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G62" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H62" s="18" t="str">
         <f ca="1">IF(F62&lt;=0, "VENDA","CAREPACK")</f>
@@ -4149,9 +4149,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:15">
       <c r="A63" s="30" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>15</v>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="E63" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F63" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G63" s="16" t="s">
         <v>66</v>
@@ -4193,9 +4193,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:15">
       <c r="A64" s="31" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B64" s="27" t="s">
         <v>15</v>
@@ -4208,11 +4208,11 @@
       </c>
       <c r="E64" s="23">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F64" s="24">
         <f t="shared" ca="1" si="5"/>
-        <v>-144</v>
+        <v>-145</v>
       </c>
       <c r="G64" s="25" t="s">
         <v>16</v>
@@ -4237,9 +4237,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:15">
       <c r="A65" s="30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B65" s="20" t="s">
         <v>20</v>
@@ -4252,11 +4252,11 @@
       </c>
       <c r="E65" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F65" s="15">
         <f t="shared" ca="1" si="5"/>
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G65" s="16" t="s">
         <v>63</v>
@@ -4280,9 +4280,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:15">
       <c r="A66" s="30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>15</v>
@@ -4295,11 +4295,11 @@
       </c>
       <c r="E66" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F66" s="15">
         <f t="shared" ref="F66:F68" ca="1" si="9">D66-E66</f>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G66" s="16" t="s">
         <v>31</v>
@@ -4324,9 +4324,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:15">
       <c r="A67" s="30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>15</v>
@@ -4339,11 +4339,11 @@
       </c>
       <c r="E67" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F67" s="15">
         <f t="shared" ca="1" si="9"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G67" s="16" t="s">
         <v>63</v>
@@ -4368,9 +4368,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="68" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:15" s="9" customFormat="1">
       <c r="A68" s="30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B68" s="14" t="s">
         <v>15</v>
@@ -4383,11 +4383,11 @@
       </c>
       <c r="E68" s="11">
         <f t="shared" ca="1" si="4"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F68" s="15">
         <f t="shared" ca="1" si="9"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G68" s="16" t="s">
         <v>32</v>
@@ -4412,9 +4412,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:15">
       <c r="A69" s="30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B69" s="14"/>
       <c r="C69" s="12"/>
@@ -4435,9 +4435,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:15">
       <c r="A70" s="31" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B70" s="27" t="s">
         <v>15</v>
@@ -4450,11 +4450,11 @@
       </c>
       <c r="E70" s="13">
         <f t="shared" ref="E70:E104" ca="1" si="10">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F70" s="24">
         <f t="shared" ref="F70:F104" ca="1" si="11">D70-E70</f>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G70" s="25" t="s">
         <v>22</v>
@@ -4477,9 +4477,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:15">
       <c r="A71" s="30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B71" s="20" t="s">
         <v>20</v>
@@ -4492,11 +4492,11 @@
       </c>
       <c r="E71" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F71" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G71" s="16" t="s">
         <v>34</v>
@@ -4505,7 +4505,7 @@
         <v>35</v>
       </c>
       <c r="I71" s="18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J71" s="15" t="s">
         <v>24</v>
@@ -4514,7 +4514,7 @@
         <v>44841</v>
       </c>
       <c r="L71" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M71" s="12"/>
       <c r="N71" s="12"/>
@@ -4522,9 +4522,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:15">
       <c r="A72" s="30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B72" s="20" t="s">
         <v>20</v>
@@ -4537,11 +4537,11 @@
       </c>
       <c r="E72" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F72" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G72" s="16" t="s">
         <v>66</v>
@@ -4564,9 +4564,9 @@
       <c r="N72" s="12"/>
       <c r="O72" s="29"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:15">
       <c r="A73" s="30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B73" s="20" t="s">
         <v>20</v>
@@ -4579,11 +4579,11 @@
       </c>
       <c r="E73" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F73" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G73" s="16" t="s">
         <v>22</v>
@@ -4608,9 +4608,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="74" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:15" s="9" customFormat="1">
       <c r="A74" s="31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B74" s="22" t="s">
         <v>20</v>
@@ -4624,22 +4624,22 @@
       </c>
       <c r="H74" s="26"/>
       <c r="I74" s="26" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="J74" s="24" t="s">
         <v>18</v>
       </c>
       <c r="K74" s="13"/>
       <c r="L74" s="13" t="s">
-        <v>205</v>
+        <v>117</v>
       </c>
       <c r="M74" s="13"/>
       <c r="N74" s="13"/>
       <c r="O74" s="32"/>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:15">
       <c r="A75" s="30" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B75" s="14" t="s">
         <v>15</v>
@@ -4652,11 +4652,11 @@
       </c>
       <c r="E75" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F75" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G75" s="16" t="s">
         <v>32</v>
@@ -4675,7 +4675,7 @@
         <v>45999</v>
       </c>
       <c r="L75" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="M75" s="12"/>
       <c r="N75" s="12"/>
@@ -4683,9 +4683,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:15">
       <c r="A76" s="30" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B76" s="20" t="s">
         <v>57</v>
@@ -4698,11 +4698,11 @@
       </c>
       <c r="E76" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F76" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G76" s="16" t="s">
         <v>85</v>
@@ -4721,7 +4721,7 @@
         <v>45371</v>
       </c>
       <c r="L76" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="M76" s="12"/>
       <c r="N76" s="12"/>
@@ -4729,9 +4729,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:15">
       <c r="A77" s="30" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B77" s="14" t="s">
         <v>15</v>
@@ -4744,11 +4744,11 @@
       </c>
       <c r="E77" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F77" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G77" s="16" t="s">
         <v>23</v>
@@ -4767,7 +4767,7 @@
         <v>45273</v>
       </c>
       <c r="L77" s="12" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="M77" s="12"/>
       <c r="N77" s="12"/>
@@ -4775,9 +4775,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:15">
       <c r="A78" s="30" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B78" s="20" t="s">
         <v>51</v>
@@ -4790,20 +4790,20 @@
       </c>
       <c r="E78" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F78" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="G78" s="16" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="H78" s="18" t="s">
         <v>35</v>
       </c>
       <c r="I78" s="18" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="J78" s="15" t="s">
         <v>24</v>
@@ -4812,7 +4812,7 @@
         <v>45989</v>
       </c>
       <c r="L78" s="12" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="M78" s="12"/>
       <c r="N78" s="12"/>
@@ -4820,9 +4820,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:15">
       <c r="A79" s="30" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B79" s="14" t="s">
         <v>15</v>
@@ -4835,11 +4835,11 @@
       </c>
       <c r="E79" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F79" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G79" s="16" t="s">
         <v>34</v>
@@ -4849,7 +4849,7 @@
         <v>VENDA</v>
       </c>
       <c r="I79" s="18" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="J79" s="15" t="s">
         <v>24</v>
@@ -4864,9 +4864,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:15">
       <c r="A80" s="30" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B80" s="14" t="s">
         <v>15</v>
@@ -4879,11 +4879,11 @@
       </c>
       <c r="E80" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F80" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G80" s="16" t="s">
         <v>66</v>
@@ -4908,9 +4908,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:15">
       <c r="A81" s="30" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B81" s="14" t="s">
         <v>15</v>
@@ -4923,11 +4923,11 @@
       </c>
       <c r="E81" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F81" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G81" s="16" t="s">
         <v>26</v>
@@ -4952,9 +4952,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:15">
       <c r="A82" s="30" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B82" s="14" t="s">
         <v>15</v>
@@ -4967,11 +4967,11 @@
       </c>
       <c r="E82" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F82" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G82" s="16" t="s">
         <v>26</v>
@@ -4996,9 +4996,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:15">
       <c r="A83" s="30" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B83" s="20" t="s">
         <v>57</v>
@@ -5011,11 +5011,11 @@
       </c>
       <c r="E83" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F83" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G83" s="16" t="s">
         <v>22</v>
@@ -5040,9 +5040,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:15">
       <c r="A84" s="30" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B84" s="20" t="s">
         <v>57</v>
@@ -5055,11 +5055,11 @@
       </c>
       <c r="E84" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F84" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G84" s="16" t="s">
         <v>16</v>
@@ -5084,9 +5084,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:15">
       <c r="A85" s="30" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B85" s="14" t="s">
         <v>28</v>
@@ -5099,11 +5099,11 @@
       </c>
       <c r="E85" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F85" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G85" s="16" t="s">
         <v>75</v>
@@ -5117,7 +5117,7 @@
       <c r="J85" s="15"/>
       <c r="K85" s="12"/>
       <c r="L85" s="12" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="M85" s="12"/>
       <c r="N85" s="12"/>
@@ -5125,12 +5125,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:15">
       <c r="A86" s="30" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C86" s="12">
         <v>46082</v>
@@ -5140,11 +5140,11 @@
       </c>
       <c r="E86" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F86" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G86" s="16" t="s">
         <v>34</v>
@@ -5153,7 +5153,7 @@
         <v>35</v>
       </c>
       <c r="I86" s="18" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J86" s="15" t="s">
         <v>24</v>
@@ -5168,9 +5168,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:15">
       <c r="A87" s="30" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B87" s="20" t="s">
         <v>20</v>
@@ -5183,11 +5183,11 @@
       </c>
       <c r="E87" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F87" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G87" s="16" t="s">
         <v>73</v>
@@ -5196,7 +5196,7 @@
         <v>35</v>
       </c>
       <c r="I87" s="18" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J87" s="16" t="s">
         <v>74</v>
@@ -5211,9 +5211,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:15">
       <c r="A88" s="30" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B88" s="14" t="s">
         <v>15</v>
@@ -5226,11 +5226,11 @@
       </c>
       <c r="E88" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F88" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G88" s="16" t="s">
         <v>21</v>
@@ -5253,9 +5253,9 @@
       <c r="N88" s="12"/>
       <c r="O88" s="29"/>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:15">
       <c r="A89" s="30" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B89" s="14" t="s">
         <v>15</v>
@@ -5268,11 +5268,11 @@
       </c>
       <c r="E89" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F89" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G89" s="16" t="s">
         <v>31</v>
@@ -5297,12 +5297,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:15">
       <c r="A90" s="30" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B90" s="20" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C90" s="12">
         <v>46199</v>
@@ -5312,20 +5312,20 @@
       </c>
       <c r="E90" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F90" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G90" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H90" s="18" t="s">
         <v>35</v>
       </c>
       <c r="I90" s="18" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J90" s="15" t="s">
         <v>18</v>
@@ -5338,9 +5338,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:15">
       <c r="A91" s="30" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B91" s="20" t="s">
         <v>57</v>
@@ -5353,11 +5353,11 @@
       </c>
       <c r="E91" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F91" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G91" s="16" t="s">
         <v>22</v>
@@ -5382,9 +5382,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:15">
       <c r="A92" s="30" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B92" s="20" t="s">
         <v>57</v>
@@ -5397,11 +5397,11 @@
       </c>
       <c r="E92" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F92" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G92" s="16" t="s">
         <v>16</v>
@@ -5424,9 +5424,9 @@
       <c r="N92" s="12"/>
       <c r="O92" s="29"/>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:15">
       <c r="A93" s="30" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B93" s="14" t="s">
         <v>15</v>
@@ -5439,14 +5439,14 @@
       </c>
       <c r="E93" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F93" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H93" s="18" t="str">
         <f t="shared" ca="1" si="13"/>
@@ -5468,9 +5468,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:15">
       <c r="A94" s="31" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B94" s="22" t="s">
         <v>57</v>
@@ -5483,11 +5483,11 @@
       </c>
       <c r="E94" s="23">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F94" s="24">
         <f t="shared" ca="1" si="11"/>
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G94" s="25" t="s">
         <v>26</v>
@@ -5506,7 +5506,7 @@
         <v>45055</v>
       </c>
       <c r="L94" s="13" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="M94" s="13"/>
       <c r="N94" s="13"/>
@@ -5514,9 +5514,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:15">
       <c r="A95" s="31" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B95" s="22" t="s">
         <v>51</v>
@@ -5529,11 +5529,11 @@
       </c>
       <c r="E95" s="23">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F95" s="24">
         <f t="shared" ca="1" si="11"/>
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G95" s="25" t="s">
         <v>16</v>
@@ -5552,7 +5552,7 @@
         <v>45908</v>
       </c>
       <c r="L95" s="13" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="M95" s="13"/>
       <c r="N95" s="13"/>
@@ -5560,9 +5560,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:15">
       <c r="A96" s="30" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B96" s="14" t="s">
         <v>15</v>
@@ -5575,11 +5575,11 @@
       </c>
       <c r="E96" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F96" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G96" s="16" t="s">
         <v>31</v>
@@ -5604,9 +5604,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="97" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:15" s="9" customFormat="1">
       <c r="A97" s="31" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B97" s="22" t="s">
         <v>20</v>
@@ -5619,11 +5619,11 @@
       </c>
       <c r="E97" s="13">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F97" s="24">
         <f t="shared" ca="1" si="11"/>
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G97" s="25" t="s">
         <v>32</v>
@@ -5648,9 +5648,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="98" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:15" ht="14.25" customHeight="1">
       <c r="A98" s="30" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B98" s="14" t="s">
         <v>15</v>
@@ -5663,11 +5663,11 @@
       </c>
       <c r="E98" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F98" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G98" s="16" t="s">
         <v>21</v>
@@ -5692,9 +5692,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:15">
       <c r="A99" s="30" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B99" s="20" t="s">
         <v>57</v>
@@ -5707,11 +5707,11 @@
       </c>
       <c r="E99" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F99" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G99" s="16" t="s">
         <v>85</v>
@@ -5736,9 +5736,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:15">
       <c r="A100" s="30" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B100" s="14" t="s">
         <v>15</v>
@@ -5751,11 +5751,11 @@
       </c>
       <c r="E100" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F100" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G100" s="16" t="s">
         <v>31</v>
@@ -5780,9 +5780,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:15">
       <c r="A101" s="30" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B101" s="20" t="s">
         <v>57</v>
@@ -5795,14 +5795,14 @@
       </c>
       <c r="E101" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F101" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H101" s="18" t="str">
         <f t="shared" ca="1" si="13"/>
@@ -5824,9 +5824,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:15">
       <c r="A102" s="30" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B102" s="20" t="s">
         <v>20</v>
@@ -5839,21 +5839,21 @@
       </c>
       <c r="E102" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F102" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G102" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H102" s="18" t="str">
         <f t="shared" ca="1" si="13"/>
         <v>CAREPACK</v>
       </c>
       <c r="I102" s="18" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="J102" s="15" t="s">
         <v>18</v>
@@ -5868,9 +5868,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:15">
       <c r="A103" s="30" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B103" s="20" t="s">
         <v>57</v>
@@ -5883,11 +5883,11 @@
       </c>
       <c r="E103" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F103" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G103" s="16" t="s">
         <v>16</v>
@@ -5912,9 +5912,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="104" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:15" s="9" customFormat="1">
       <c r="A104" s="30" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B104" s="20" t="s">
         <v>57</v>
@@ -5927,14 +5927,14 @@
       </c>
       <c r="E104" s="12">
         <f t="shared" ca="1" si="10"/>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F104" s="15">
         <f t="shared" ca="1" si="11"/>
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G104" s="16" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="H104" s="18" t="str">
         <f t="shared" ca="1" si="13"/>
@@ -5956,9 +5956,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:15">
       <c r="A105" s="30" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B105" s="14" t="s">
         <v>15</v>
@@ -5981,9 +5981,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:15">
       <c r="A106" s="30" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B106" s="20" t="s">
         <v>20</v>
@@ -5996,11 +5996,11 @@
       </c>
       <c r="E106" s="12">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F106" s="15">
         <f ca="1">D106-E106</f>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G106" s="16" t="s">
         <v>38</v>
@@ -6023,9 +6023,9 @@
       <c r="N106" s="12"/>
       <c r="O106" s="29"/>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:15">
       <c r="A107" s="30" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B107" s="20" t="s">
         <v>20</v>
@@ -6038,11 +6038,11 @@
       </c>
       <c r="E107" s="12">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F107" s="15">
         <f ca="1">D107-E107</f>
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="G107" s="16" t="s">
         <v>29</v>
@@ -6067,9 +6067,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:15">
       <c r="A108" s="30" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B108" s="20" t="s">
         <v>20</v>
@@ -6082,11 +6082,11 @@
       </c>
       <c r="E108" s="12">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F108" s="15">
         <f ca="1">D108-E108</f>
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G108" s="16" t="s">
         <v>34</v>
@@ -6111,9 +6111,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:15">
       <c r="A109" s="30" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B109" s="14" t="s">
         <v>15</v>
@@ -6126,14 +6126,14 @@
       </c>
       <c r="E109" s="12">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F109" s="15">
         <f ca="1">D109-E109</f>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H109" s="18" t="str">
         <f ca="1">IF(F109&lt;=0, "VENDA","CAREPACK")</f>
@@ -6155,9 +6155,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="110" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:15" ht="15" thickBot="1">
       <c r="A110" s="33" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B110" s="34" t="s">
         <v>15</v>
@@ -6170,11 +6170,11 @@
       </c>
       <c r="E110" s="35">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F110" s="37">
         <f ca="1">D110-E110</f>
-        <v>-2030</v>
+        <v>-2031</v>
       </c>
       <c r="G110" s="38" t="s">
         <v>31</v>
@@ -6212,25 +6212,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C0B4294-6308-408D-A7E0-6148B7D61ACB}">
   <dimension ref="A1:N38"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="28.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="9.7265625" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" customWidth="1"/>
     <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.26953125" style="7" customWidth="1"/>
-    <col min="9" max="9" width="15.54296875" style="7" customWidth="1"/>
-    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" style="7" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="7" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="4" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6238,10 +6238,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>4</v>
@@ -6259,27 +6259,27 @@
         <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C2" s="3">
         <v>45670</v>
@@ -6290,14 +6290,14 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I2" s="6"/>
       <c r="J2" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K2" s="3">
         <v>45670</v>
@@ -6312,12 +6312,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C3" s="3">
         <v>45670</v>
@@ -6328,14 +6328,14 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K3" s="3">
         <v>45685</v>
@@ -6350,12 +6350,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14">
       <c r="A4" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C4" s="3">
         <v>45670</v>
@@ -6366,14 +6366,14 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I4" s="6"/>
       <c r="J4" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K4" s="3">
         <v>45670</v>
@@ -6388,12 +6388,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C5" s="3">
         <v>45670</v>
@@ -6404,14 +6404,14 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K5" s="3">
         <v>45670</v>
@@ -6426,12 +6426,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14">
       <c r="A6" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C6" s="3">
         <v>44866</v>
@@ -6442,14 +6442,14 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I6" s="6"/>
       <c r="J6" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K6" s="3">
         <v>42867</v>
@@ -6464,12 +6464,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14">
       <c r="A7" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C7" s="3">
         <v>45670</v>
@@ -6480,14 +6480,14 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I7" s="6"/>
       <c r="J7" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K7" s="3">
         <v>45670</v>
@@ -6502,12 +6502,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14">
       <c r="A8" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C8" s="3">
         <v>45670</v>
@@ -6518,14 +6518,14 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I8" s="6"/>
       <c r="J8" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K8" s="3">
         <v>45670</v>
@@ -6540,12 +6540,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14">
       <c r="A9" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C9" s="3">
         <v>45670</v>
@@ -6556,14 +6556,14 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K9" s="3">
         <v>45670</v>
@@ -6578,12 +6578,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14">
       <c r="A10" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C10" s="3">
         <v>44501</v>
@@ -6594,14 +6594,14 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I10" s="6"/>
       <c r="J10" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K10" s="3">
         <v>42949</v>
@@ -6616,12 +6616,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14">
       <c r="A11" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C11" s="3">
         <v>45670</v>
@@ -6632,14 +6632,14 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I11" s="6"/>
       <c r="J11" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K11" s="3">
         <v>45670</v>
@@ -6654,12 +6654,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14">
       <c r="A12" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C12" s="3">
         <v>45670</v>
@@ -6670,14 +6670,14 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I12" s="6"/>
       <c r="J12" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K12" s="3">
         <v>45670</v>
@@ -6692,12 +6692,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14">
       <c r="A13" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C13" s="3">
         <v>45658</v>
@@ -6708,14 +6708,14 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I13" s="6"/>
       <c r="J13" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K13" s="3">
         <v>42972</v>
@@ -6730,12 +6730,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14">
       <c r="A14" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C14" s="3">
         <v>45670</v>
@@ -6746,14 +6746,14 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I14" s="6"/>
       <c r="J14" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K14" s="3">
         <v>45670</v>
@@ -6768,12 +6768,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14">
       <c r="A15" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C15" s="3">
         <v>44911</v>
@@ -6784,14 +6784,14 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K15" s="3">
         <v>41417</v>
@@ -6806,12 +6806,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14">
       <c r="A16" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C16" s="3">
         <v>45670</v>
@@ -6822,14 +6822,14 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I16" s="6"/>
       <c r="J16" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K16" s="3">
         <v>45670</v>
@@ -6844,12 +6844,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14">
       <c r="A17" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C17" s="3">
         <v>45670</v>
@@ -6860,14 +6860,14 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K17" s="3">
         <v>45670</v>
@@ -6882,12 +6882,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14">
       <c r="A18" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C18" s="3">
         <v>45670</v>
@@ -6898,14 +6898,14 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K18" s="3">
         <v>45670</v>
@@ -6920,12 +6920,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14">
       <c r="A19" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C19" s="3">
         <v>45670</v>
@@ -6936,14 +6936,14 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K19" s="3">
         <v>45670</v>
@@ -6958,12 +6958,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14">
       <c r="A20" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C20" s="3">
         <v>45670</v>
@@ -6974,14 +6974,14 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I20" s="6"/>
       <c r="J20" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K20" s="3">
         <v>45670</v>
@@ -6996,12 +6996,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14">
       <c r="A21" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C21" s="3">
         <v>45658</v>
@@ -7012,14 +7012,14 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K21" s="3">
         <v>40396</v>
@@ -7034,12 +7034,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14">
       <c r="A22" s="2" t="s">
         <v>87</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C22" s="3">
         <v>45658</v>
@@ -7050,14 +7050,14 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I22" s="6"/>
       <c r="J22" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K22" s="3">
         <v>43783</v>
@@ -7072,12 +7072,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14">
       <c r="A23" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C23" s="3">
         <v>44501</v>
@@ -7088,14 +7088,14 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K23" s="3">
         <v>42119</v>
@@ -7110,12 +7110,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14">
       <c r="A24" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C24" s="3">
         <v>45670</v>
@@ -7126,14 +7126,14 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I24" s="6"/>
       <c r="J24" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K24" s="3">
         <v>45670</v>
@@ -7148,12 +7148,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14">
       <c r="A25" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C25" s="3">
         <v>45670</v>
@@ -7164,14 +7164,14 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
       <c r="G25" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I25" s="6"/>
       <c r="J25" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K25" s="3">
         <v>45670</v>
@@ -7186,12 +7186,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14">
       <c r="A26" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C26" s="3">
         <v>45670</v>
@@ -7202,14 +7202,14 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I26" s="6"/>
       <c r="J26" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K26" s="3">
         <v>45670</v>
@@ -7224,12 +7224,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14">
       <c r="A27" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C27" s="3">
         <v>45670</v>
@@ -7240,14 +7240,14 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I27" s="6"/>
       <c r="J27" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K27" s="3">
         <v>45670</v>
@@ -7262,12 +7262,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14">
       <c r="A28" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C28" s="3">
         <v>45658</v>
@@ -7278,14 +7278,14 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I28" s="6"/>
       <c r="J28" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K28" s="3">
         <v>39766</v>
@@ -7300,12 +7300,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14">
       <c r="A29" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C29" s="3">
         <v>45658</v>
@@ -7316,14 +7316,14 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I29" s="6"/>
       <c r="J29" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K29" s="3">
         <v>41075</v>
@@ -7338,12 +7338,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14">
       <c r="A30" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C30" s="3">
         <v>45670</v>
@@ -7354,14 +7354,14 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I30" s="6"/>
       <c r="J30" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K30" s="3">
         <v>45670</v>
@@ -7376,12 +7376,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14">
       <c r="A31" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C31" s="3">
         <v>45670</v>
@@ -7392,14 +7392,14 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K31" s="3">
         <v>45670</v>
@@ -7414,12 +7414,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14">
       <c r="A32" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C32" s="3">
         <v>45016</v>
@@ -7430,14 +7430,14 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I32" s="6"/>
       <c r="J32" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K32" s="3">
         <v>45016</v>
@@ -7452,12 +7452,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14">
       <c r="A33" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C33" s="3">
         <v>44743</v>
@@ -7468,14 +7468,14 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I33" s="6"/>
       <c r="J33" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K33" s="3">
         <v>42886</v>
@@ -7490,12 +7490,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:14">
       <c r="A34" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C34" s="3">
         <v>45670</v>
@@ -7506,14 +7506,14 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K34" s="3">
         <v>45670</v>
@@ -7528,12 +7528,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14">
       <c r="A35" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C35" s="3">
         <v>45009</v>
@@ -7544,14 +7544,14 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K35" s="3">
         <v>45009</v>
@@ -7566,12 +7566,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:14">
       <c r="A36" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C36" s="3">
         <v>45658</v>
@@ -7582,14 +7582,14 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I36" s="6"/>
       <c r="J36" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K36" s="3">
         <v>43021</v>
@@ -7604,12 +7604,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:14">
       <c r="A37" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C37" s="3">
         <v>45670</v>
@@ -7620,14 +7620,14 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I37" s="6"/>
       <c r="J37" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K37" s="3">
         <v>45670</v>
@@ -7642,12 +7642,12 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:14">
       <c r="A38" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C38" s="3">
         <v>44866</v>
@@ -7658,14 +7658,14 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I38" s="6"/>
       <c r="J38" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K38" s="3">
         <v>40389</v>

</xml_diff>